<commit_message>
Actualizacion automatica SIPREM y Casuistica
</commit_message>
<xml_diff>
--- a/siprem_latest.xlsx
+++ b/siprem_latest.xlsx
@@ -29,7 +29,7 @@
     <t>FECHA</t>
   </si>
   <si>
-    <t>23/10/2026 a las 07:57:27</t>
+    <t>23/10/2026 a las 08:01:08</t>
   </si>
   <si>
     <t>Num_Lote</t>
@@ -26141,7 +26141,7 @@
         <v>1000</v>
       </c>
       <c r="B240" s="4" t="s">
-        <v>454</v>
+        <v>201</v>
       </c>
       <c r="C240" s="4">
         <v>169948127</v>
@@ -26199,7 +26199,7 @@
         <v>2</v>
       </c>
       <c r="X240" s="4" t="s">
-        <v>70</v>
+        <v>192</v>
       </c>
       <c r="Y240" s="4"/>
       <c r="Z240" s="4" t="s">

</xml_diff>